<commit_message>
Finished dbt config and started build on event classification, location and date dimensions.
</commit_message>
<xml_diff>
--- a/model_analysis.xlsx
+++ b/model_analysis.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EdwardCoates\Dev\snowflake_sandbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64E7E9C6-D84A-4E1A-8E75-AF4F74445559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C97D4CDE-1D4E-4354-ADEC-41BCD49F6EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0818FD26-D4B8-4367-BAC1-03867A914A11}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{0818FD26-D4B8-4367-BAC1-03867A914A11}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="1. Data Dictionary" sheetId="4" r:id="rId1"/>
+    <sheet name="2. Data Model" sheetId="3" r:id="rId2"/>
+    <sheet name="3. Raw Data" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="350">
   <si>
     <t>ID</t>
   </si>
@@ -131,6 +133,9 @@
     <t>DEPTH</t>
   </si>
   <si>
+    <t>DWH_CREATE_TIMESTAMP</t>
+  </si>
+  <si>
     <t>us6000tahc</t>
   </si>
   <si>
@@ -270,13 +275,834 @@
   </si>
   <si>
     <t>M 5.0 - 106 km NW of Coquimbo, Chile</t>
+  </si>
+  <si>
+    <t>GeoJSON Source Path</t>
+  </si>
+  <si>
+    <t>Data Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Event ID</t>
+  </si>
+  <si>
+    <t>feature.id</t>
+  </si>
+  <si>
+    <t>Unique preferred identifier for the event (e.g. us6000tahc), formed from the preferred network + code.</t>
+  </si>
+  <si>
+    <t>Natural / business key. The 'preferred' id can change over time — see IDS for all aliases.</t>
+  </si>
+  <si>
+    <t>Magnitude</t>
+  </si>
+  <si>
+    <t>properties.mag</t>
+  </si>
+  <si>
+    <t>Size of the event on the scale named in MAGTYPE.</t>
+  </si>
+  <si>
+    <t>Logarithmic → NON-ADDITIVE. Never SUM; use MIN/MAX/AVG/COUNT.</t>
+  </si>
+  <si>
+    <t>Location Description</t>
+  </si>
+  <si>
+    <t>properties.place</t>
+  </si>
+  <si>
+    <t>Human-readable region, usually 'distance + direction of + named place, country', e.g. '56 km W of La Ligua, Chile'.</t>
+  </si>
+  <si>
+    <t>Semi-structured. Parse into distance / direction / nearest place / country. Some values are bare region names.</t>
+  </si>
+  <si>
+    <t>Origin Time (UTC)</t>
+  </si>
+  <si>
+    <t>properties.time</t>
+  </si>
+  <si>
+    <t>When rupture began (the 'origin' time), in milliseconds since 1970-01-01 UTC (no leap seconds).</t>
+  </si>
+  <si>
+    <t>Divide by 1000 before casting to timestamp. This is the anchor for the DATE dimension.</t>
+  </si>
+  <si>
+    <t>Last Updated Time (UTC)</t>
+  </si>
+  <si>
+    <t>properties.updated</t>
+  </si>
+  <si>
+    <t>When this event record was last modified by USGS.</t>
+  </si>
+  <si>
+    <t>Use as the change indicator for CDC / restated facts. Same epoch-ms handling as TIME.</t>
+  </si>
+  <si>
+    <t>Timezone Offset (min)</t>
+  </si>
+  <si>
+    <t>properties.tz</t>
+  </si>
+  <si>
+    <t>Historical timezone offset from UTC (minutes) at the epicentre.</t>
+  </si>
+  <si>
+    <t>DEPRECATED — almost always null (blank in the sample). Safe to drop.</t>
+  </si>
+  <si>
+    <t>Event Page URL</t>
+  </si>
+  <si>
+    <t>properties.url</t>
+  </si>
+  <si>
+    <t>Link to the human-readable USGS event page.</t>
+  </si>
+  <si>
+    <t>Degenerate attribute — keep on the fact, do not build a dimension for it.</t>
+  </si>
+  <si>
+    <t>Detail Feed URL</t>
+  </si>
+  <si>
+    <t>properties.detail</t>
+  </si>
+  <si>
+    <t>Link to the GeoJSON detail feed (full product suite) for the event.</t>
+  </si>
+  <si>
+    <t>Degenerate; useful as an API drill-through path.</t>
+  </si>
+  <si>
+    <t>Felt Reports Count</t>
+  </si>
+  <si>
+    <t>properties.felt</t>
+  </si>
+  <si>
+    <t>Number of 'Did You Feel It?' (DYFI) responses submitted for the event.</t>
+  </si>
+  <si>
+    <t>Null = no reports. This is the one clearly ADDITIVE measure.</t>
+  </si>
+  <si>
+    <t>Max Reported Intensity (CDI)</t>
+  </si>
+  <si>
+    <t>properties.cdi</t>
+  </si>
+  <si>
+    <t>Maximum community-determined intensity (Modified Mercalli) from DYFI reports.</t>
+  </si>
+  <si>
+    <t>Non-additive. Null when there are no felt reports.</t>
+  </si>
+  <si>
+    <t>Max Estimated Intensity (MMI)</t>
+  </si>
+  <si>
+    <t>properties.mmi</t>
+  </si>
+  <si>
+    <t>Maximum estimated instrumental intensity (Modified Mercalli) from ShakeMap.</t>
+  </si>
+  <si>
+    <t>Non-additive. Pairs with CDI (reported vs modelled shaking).</t>
+  </si>
+  <si>
+    <t>PAGER Alert Level</t>
+  </si>
+  <si>
+    <t>properties.alert</t>
+  </si>
+  <si>
+    <t>PAGER impact alert colour: green / yellow / orange / red.</t>
+  </si>
+  <si>
+    <t>Null = not assessed → map to 'none'. Ordinal severity.</t>
+  </si>
+  <si>
+    <t>Review Status</t>
+  </si>
+  <si>
+    <t>properties.status</t>
+  </si>
+  <si>
+    <t>'automatic' (posted by machine) or 'reviewed' (checked by a human).</t>
+  </si>
+  <si>
+    <t>Can change over an event's life → candidate for slowly-changing tracking.</t>
+  </si>
+  <si>
+    <t>Tsunami Flag</t>
+  </si>
+  <si>
+    <t>properties.tsunami</t>
+  </si>
+  <si>
+    <t>1 for events in oceanic regions that could generate a tsunami; otherwise 0.</t>
+  </si>
+  <si>
+    <t>A flag, not a confirmed warning. Cast 0/1 → boolean.</t>
+  </si>
+  <si>
+    <t>Significance</t>
+  </si>
+  <si>
+    <t>properties.sig</t>
+  </si>
+  <si>
+    <t>0–1000 composite score from magnitude, max MMI, felt reports and estimated impact. Higher = more significant.</t>
+  </si>
+  <si>
+    <t>Non-additive.</t>
+  </si>
+  <si>
+    <t>Preferred Network</t>
+  </si>
+  <si>
+    <t>properties.net</t>
+  </si>
+  <si>
+    <t>ID of the contributor whose solution is preferred (e.g. us, nc, ci, ak).</t>
+  </si>
+  <si>
+    <t>Combine with CODE to reconstruct the id. Good basis for a source dimension.</t>
+  </si>
+  <si>
+    <t>Network Event Code</t>
+  </si>
+  <si>
+    <t>properties.code</t>
+  </si>
+  <si>
+    <t>Identifier assigned to the event by the preferred network.</t>
+  </si>
+  <si>
+    <t>net + code ≈ id.</t>
+  </si>
+  <si>
+    <t>Associated IDs</t>
+  </si>
+  <si>
+    <t>properties.ids</t>
+  </si>
+  <si>
+    <t>Comma-wrapped list of every event id associated with this event.</t>
+  </si>
+  <si>
+    <t>Trim leading/trailing commas, then split. Multi-valued → bridge table.</t>
+  </si>
+  <si>
+    <t>Contributing Sources</t>
+  </si>
+  <si>
+    <t>properties.sources</t>
+  </si>
+  <si>
+    <t>Comma-wrapped list of networks that contributed data to the event.</t>
+  </si>
+  <si>
+    <t>Multi-valued → bridge table (BRG_EVENT_SOURCES).</t>
+  </si>
+  <si>
+    <t>Product Types</t>
+  </si>
+  <si>
+    <t>properties.types</t>
+  </si>
+  <si>
+    <t>Comma-wrapped list of products available (dyfi, shakemap, moment-tensor, origin, phase-data ...).</t>
+  </si>
+  <si>
+    <t>Multi-valued → bridge table (BRG_EVENT_PRODUCT_TYPES).</t>
+  </si>
+  <si>
+    <t>Stations Used</t>
+  </si>
+  <si>
+    <t>properties.nst</t>
+  </si>
+  <si>
+    <t>Number of seismic stations used to locate the event.</t>
+  </si>
+  <si>
+    <t>Data-quality metric. Treat as non-additive.</t>
+  </si>
+  <si>
+    <t>Nearest Station Distance (°)</t>
+  </si>
+  <si>
+    <t>properties.dmin</t>
+  </si>
+  <si>
+    <t>Horizontal distance from epicentre to the nearest station, in degrees (1° ≈ 111.2 km). Smaller = more reliable depth.</t>
+  </si>
+  <si>
+    <t>Quality metric; non-additive.</t>
+  </si>
+  <si>
+    <t>Travel-time Residual (s)</t>
+  </si>
+  <si>
+    <t>properties.rms</t>
+  </si>
+  <si>
+    <t>Root-mean-square of travel-time residuals, in seconds. Lower = better fit.</t>
+  </si>
+  <si>
+    <t>Azimuthal Gap (°)</t>
+  </si>
+  <si>
+    <t>properties.gap</t>
+  </si>
+  <si>
+    <t>Largest azimuthal gap between adjacent stations, in degrees. Below 180° is preferred.</t>
+  </si>
+  <si>
+    <t>Magnitude Type</t>
+  </si>
+  <si>
+    <t>properties.magType</t>
+  </si>
+  <si>
+    <t>Method used to compute MAG (mb, mww, ml, md, ms ...).</t>
+  </si>
+  <si>
+    <t>Decode via a lookup. Meaningless without MAG.</t>
+  </si>
+  <si>
+    <t>Event Type</t>
+  </si>
+  <si>
+    <t>properties.type</t>
+  </si>
+  <si>
+    <t>Class of seismic event: earthquake, quarry blast, explosion, ice quake, etc.</t>
+  </si>
+  <si>
+    <t>Low cardinality → natural dimension attribute.</t>
+  </si>
+  <si>
+    <t>Event Title</t>
+  </si>
+  <si>
+    <t>properties.title</t>
+  </si>
+  <si>
+    <t>Display title, e.g. 'M 5.1 - 56 km W of La Ligua, Chile'.</t>
+  </si>
+  <si>
+    <t>Redundant — derivable from MAG + PLACE. Drop, or keep as a degenerate label.</t>
+  </si>
+  <si>
+    <t>Longitude (°)</t>
+  </si>
+  <si>
+    <t>geometry.coordinates[0]</t>
+  </si>
+  <si>
+    <t>Epicentre longitude. Negative = west of Greenwich.</t>
+  </si>
+  <si>
+    <t>Event-grain coordinate → stays on the fact.</t>
+  </si>
+  <si>
+    <t>Latitude (°)</t>
+  </si>
+  <si>
+    <t>geometry.coordinates[1]</t>
+  </si>
+  <si>
+    <t>Epicentre latitude. Negative = southern hemisphere.</t>
+  </si>
+  <si>
+    <t>Depth (km)</t>
+  </si>
+  <si>
+    <t>geometry.coordinates[2]</t>
+  </si>
+  <si>
+    <t>Focal depth below the surface, in kilometres.</t>
+  </si>
+  <si>
+    <t>Non-additive measure.</t>
+  </si>
+  <si>
+    <t>Source Heading</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>FACT_SEISMIC_EVENT</t>
+  </si>
+  <si>
+    <t>DIM_DATE</t>
+  </si>
+  <si>
+    <t>DIM_LOCATION</t>
+  </si>
+  <si>
+    <t>DIM_EVENT_CLASSIFICATION</t>
+  </si>
+  <si>
+    <t>DIM_ALERT_STATUS</t>
+  </si>
+  <si>
+    <t>Fact table. Grain: one row per earthquake event. Holds dimension FKs, degenerates and measures.</t>
+  </si>
+  <si>
+    <t>Conformed calendar dimension, one row per day.</t>
+  </si>
+  <si>
+    <t>Geography dimension, one row per distinct named region.</t>
+  </si>
+  <si>
+    <t>Classification dimension, one row per event type + magnitude type + magnitude band, with codes decoded to readable values.</t>
+  </si>
+  <si>
+    <t>Junk dimension, one row per valid combination of pager alert level, review status, tsunami flag and felt-reports flag.</t>
+  </si>
+  <si>
+    <t>EVENT_ID</t>
+  </si>
+  <si>
+    <t>DATE_KEY</t>
+  </si>
+  <si>
+    <t>DIRECTION_FROM_PLACE</t>
+  </si>
+  <si>
+    <t>EVENT_URL</t>
+  </si>
+  <si>
+    <t>DETAIL_URL</t>
+  </si>
+  <si>
+    <t>DEPTH_KM</t>
+  </si>
+  <si>
+    <t>MAGNITUDE</t>
+  </si>
+  <si>
+    <t>DISTANCE_FROM_PLACE_KM</t>
+  </si>
+  <si>
+    <t>FELT_COUNT</t>
+  </si>
+  <si>
+    <t>CDI_MAX</t>
+  </si>
+  <si>
+    <t>MMI_MAX</t>
+  </si>
+  <si>
+    <t>SIGNIFICANCE</t>
+  </si>
+  <si>
+    <t>NUM_STATIONS</t>
+  </si>
+  <si>
+    <t>DMIN_DEG</t>
+  </si>
+  <si>
+    <t>RMS_SEC</t>
+  </si>
+  <si>
+    <t>AZIMUTHAL_GAP_DEG</t>
+  </si>
+  <si>
+    <t>EVENT_KEY</t>
+  </si>
+  <si>
+    <t>LOCATION_KEY</t>
+  </si>
+  <si>
+    <t>EVENT_CLASS_KEY</t>
+  </si>
+  <si>
+    <t>ALERT_STATUS_KEY</t>
+  </si>
+  <si>
+    <t>INT</t>
+  </si>
+  <si>
+    <t>PK</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Calendar date.</t>
+  </si>
+  <si>
+    <t>1–31.</t>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>Monday … Sunday.</t>
+  </si>
+  <si>
+    <t>1 = Monday … 7 = Sunday.</t>
+  </si>
+  <si>
+    <t>BOOLEAN</t>
+  </si>
+  <si>
+    <t>True for Sat/Sun.</t>
+  </si>
+  <si>
+    <t>ISO week number.</t>
+  </si>
+  <si>
+    <t>1–12.</t>
+  </si>
+  <si>
+    <t>January … December.</t>
+  </si>
+  <si>
+    <t>1–4.</t>
+  </si>
+  <si>
+    <t>Calendar year.</t>
+  </si>
+  <si>
+    <t>YYYY-MM for easy grouping.</t>
+  </si>
+  <si>
+    <t>DAY_OF_MONTH</t>
+  </si>
+  <si>
+    <t>DAY_NAME</t>
+  </si>
+  <si>
+    <t>DAY_OF_WEEK_ISO</t>
+  </si>
+  <si>
+    <t>IS_WEEKEND</t>
+  </si>
+  <si>
+    <t>ISO_WEEK</t>
+  </si>
+  <si>
+    <t>MONTH_NUMBER</t>
+  </si>
+  <si>
+    <t>MONTH_NAME</t>
+  </si>
+  <si>
+    <t>QUARTER</t>
+  </si>
+  <si>
+    <t>YEAR</t>
+  </si>
+  <si>
+    <t>YEAR_MONTH</t>
+  </si>
+  <si>
+    <t>BIGINT</t>
+  </si>
+  <si>
+    <t>Surrogate key.</t>
+  </si>
+  <si>
+    <t>Named place parsed from PLACE (e.g. La Ligua).</t>
+  </si>
+  <si>
+    <t>Trailing token of PLACE (e.g. Chile, Tonga).</t>
+  </si>
+  <si>
+    <t>Populated when the region token is a US state; else null.</t>
+  </si>
+  <si>
+    <t>CHAR(1)</t>
+  </si>
+  <si>
+    <t>N or S from latitude sign.</t>
+  </si>
+  <si>
+    <t>E or W from longitude sign.</t>
+  </si>
+  <si>
+    <t>Original PLACE text, kept for audit.</t>
+  </si>
+  <si>
+    <t>US_STATE</t>
+  </si>
+  <si>
+    <t>LAT_HEMISPHERE</t>
+  </si>
+  <si>
+    <t>LON_HEMISPHERE</t>
+  </si>
+  <si>
+    <t>PLACE_RAW</t>
+  </si>
+  <si>
+    <t>earthquake / quarry blast / explosion … (TYPE).</t>
+  </si>
+  <si>
+    <t>mb, mww, ml, md … (MAGTYPE).</t>
+  </si>
+  <si>
+    <t>Decoded name (e.g. mb = short-period body-wave).</t>
+  </si>
+  <si>
+    <t>EVENT_TYPE</t>
+  </si>
+  <si>
+    <t>MAGNITUDE_TYPE_CODE</t>
+  </si>
+  <si>
+    <t>MAGNITUDE_TYPE_DESC</t>
+  </si>
+  <si>
+    <t>MAGNITUDE_BAND</t>
+  </si>
+  <si>
+    <t>Banded from MAG: Light / Moderate / Strong / Major / Great.
+5.0 - 5.9 = Moderate
+6.0 - 6.9 = Strong
+7.0 - 7.9 = Major
+8.0 - 8.9 = Great
+9.0 - 9.9 = Extreme</t>
+  </si>
+  <si>
+    <t>PAGER_ALERT_LEVEL</t>
+  </si>
+  <si>
+    <t>PAGER_ALERT_RANK</t>
+  </si>
+  <si>
+    <t>REVIEW_STATUS</t>
+  </si>
+  <si>
+    <t>IS_REVIEWED</t>
+  </si>
+  <si>
+    <t>TSUNAMI_FLAG</t>
+  </si>
+  <si>
+    <t>HAS_FELT_REPORTS</t>
+  </si>
+  <si>
+    <t>INTEGER</t>
+  </si>
+  <si>
+    <t>none / green / yellow / orange / red (ALERT).</t>
+  </si>
+  <si>
+    <t>Ordinal 0–4 for sorting/severity.</t>
+  </si>
+  <si>
+    <t>automatic / reviewed (STATUS).</t>
+  </si>
+  <si>
+    <t>True when reviewed by a human.</t>
+  </si>
+  <si>
+    <t>True when TSUNAMI = 1.</t>
+  </si>
+  <si>
+    <t>True when FELT is present and &gt; 0.</t>
+  </si>
+  <si>
+    <t>Surrogate key for each flag combination.</t>
+  </si>
+  <si>
+    <t>Surrogate PK</t>
+  </si>
+  <si>
+    <t>Surrogate primary key for the fact row.</t>
+  </si>
+  <si>
+    <t>Degenerate dim</t>
+  </si>
+  <si>
+    <t>Natural key from ID (e.g. us6000tahc).</t>
+  </si>
+  <si>
+    <t>FK → DIM_DATE</t>
+  </si>
+  <si>
+    <t>Origin date (UTC) as YYYYMMDD.</t>
+  </si>
+  <si>
+    <t>FK → DIM_LOCATION</t>
+  </si>
+  <si>
+    <t>Named-region geography of the epicentre.</t>
+  </si>
+  <si>
+    <t>FK → DIM_EVENT_CLASSIFICATION</t>
+  </si>
+  <si>
+    <t>Event type + magnitude type.</t>
+  </si>
+  <si>
+    <t>FK → DIM_ALERT_STATUS</t>
+  </si>
+  <si>
+    <t>Low-cardinality flags (junk dimension).</t>
+  </si>
+  <si>
+    <t>Degenerate</t>
+  </si>
+  <si>
+    <t>Precise origin timestamp (keeps sub-day detail).</t>
+  </si>
+  <si>
+    <t>Compass bearing parsed from PLACE (e.g. W, ESE).</t>
+  </si>
+  <si>
+    <t>USGS event page (URL).</t>
+  </si>
+  <si>
+    <t>GeoJSON detail feed (DETAIL).</t>
+  </si>
+  <si>
+    <t>DECIMAL(9,4)</t>
+  </si>
+  <si>
+    <t>Measure</t>
+  </si>
+  <si>
+    <t>Epicentre latitude.</t>
+  </si>
+  <si>
+    <t>Epicentre longitude.</t>
+  </si>
+  <si>
+    <t>DECIMAL(7,3)</t>
+  </si>
+  <si>
+    <t>Measure (non-add)</t>
+  </si>
+  <si>
+    <t>Focal depth in km.</t>
+  </si>
+  <si>
+    <t>DECIMAL(4,2)</t>
+  </si>
+  <si>
+    <t>Event magnitude — NEVER sum.</t>
+  </si>
+  <si>
+    <t>DECIMAL(7,2)</t>
+  </si>
+  <si>
+    <t>Distance to named place, parsed from PLACE.</t>
+  </si>
+  <si>
+    <t>Measure (additive)</t>
+  </si>
+  <si>
+    <t>DYFI felt-report count (FELT).</t>
+  </si>
+  <si>
+    <t>DECIMAL(3,1)</t>
+  </si>
+  <si>
+    <t>Max reported intensity (CDI).</t>
+  </si>
+  <si>
+    <t>Max estimated intensity (MMI).</t>
+  </si>
+  <si>
+    <t>Significance score 0–1000 (SIG).</t>
+  </si>
+  <si>
+    <t>Measure (quality)</t>
+  </si>
+  <si>
+    <t>Stations used (NST).</t>
+  </si>
+  <si>
+    <t>DECIMAL(7,4)</t>
+  </si>
+  <si>
+    <t>Nearest-station distance in degrees (DMIN).</t>
+  </si>
+  <si>
+    <t>DECIMAL(5,2)</t>
+  </si>
+  <si>
+    <t>Travel-time residual RMS (RMS).</t>
+  </si>
+  <si>
+    <t>DECIMAL(5,1)</t>
+  </si>
+  <si>
+    <t>Largest azimuthal gap (GAP).</t>
+  </si>
+  <si>
+    <t>DWH_UPDATE_TIMESTAMP</t>
+  </si>
+  <si>
+    <t>TIMESTAMP_NTZ(9)</t>
+  </si>
+  <si>
+    <t>Row creation date.</t>
+  </si>
+  <si>
+    <t>Row updated date.</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>EVENT_TIMESTAMP</t>
+  </si>
+  <si>
+    <t>COUNTRY</t>
+  </si>
+  <si>
+    <t>US_STATE_CODE</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>BK</t>
+  </si>
+  <si>
+    <t>REGION</t>
+  </si>
+  <si>
+    <t>Removed</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,16 +1110,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -301,22 +1152,127 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBBBBBB"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBBBBBB"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBBBBBB"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBBBBBB"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{81658078-8082-4332-9FAA-2FF5D0F440E5}">
+      <tableStyleElement type="secondRowStripe" dxfId="2"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -326,6 +1282,36 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3401880D-A971-46E3-AB92-F9A2A97672D2}" name="Table2" displayName="Table2" ref="A1:E31" totalsRowShown="0">
+  <autoFilter ref="A1:E31" xr:uid="{3401880D-A971-46E3-AB92-F9A2A97672D2}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{26C81EAB-4E14-4606-B26F-BF4BE6C8A043}" name="Source Heading"/>
+    <tableColumn id="2" xr3:uid="{5067F62A-A241-4844-A2AB-1CA8D803AB42}" name="Meaning"/>
+    <tableColumn id="3" xr3:uid="{0E2C65D7-7F24-4543-834C-ABD5FAAB89BE}" name="GeoJSON Source Path"/>
+    <tableColumn id="4" xr3:uid="{64C26296-10DF-4B50-9292-175714A1389D}" name="Description"/>
+    <tableColumn id="5" xr3:uid="{26F53C0F-A9EB-4EE3-B69D-5EFFE9978A06}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}" name="Table3" displayName="Table3" ref="A8:G72" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A8:G72" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{5D127818-973C-4145-B700-33EA8DCCBA9C}" name="Table"/>
+    <tableColumn id="2" xr3:uid="{64F6B203-BA28-42A1-8A8E-83B001CBB1A7}" name="Column"/>
+    <tableColumn id="3" xr3:uid="{1825CAC1-A664-4B19-A9AC-E5DDBAABC718}" name="Data Type"/>
+    <tableColumn id="6" xr3:uid="{5F8BC79B-72EC-4305-9B2A-02DFBDC70F87}" name="Key" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{BA7C6754-B81D-462D-B702-76D7FE5CCA61}" name="Description"/>
+    <tableColumn id="5" xr3:uid="{1B3397A1-0DFA-47D5-8B3C-420F11293C9F}" name="Notes"/>
+    <tableColumn id="7" xr3:uid="{3959C987-FF37-4778-AECC-4B8DF64B4F07}" name="Column1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -644,139 +1630,1958 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1A630FB-A618-42DB-96FD-BC7A66867678}">
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="93.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="89.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" t="s">
+        <v>131</v>
+      </c>
+      <c r="E14" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C19" t="s">
+        <v>150</v>
+      </c>
+      <c r="D19" t="s">
+        <v>151</v>
+      </c>
+      <c r="E19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20" t="s">
+        <v>154</v>
+      </c>
+      <c r="D20" t="s">
+        <v>155</v>
+      </c>
+      <c r="E20" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>157</v>
+      </c>
+      <c r="C21" t="s">
+        <v>158</v>
+      </c>
+      <c r="D21" t="s">
+        <v>159</v>
+      </c>
+      <c r="E21" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>161</v>
+      </c>
+      <c r="C22" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" t="s">
+        <v>166</v>
+      </c>
+      <c r="D23" t="s">
+        <v>167</v>
+      </c>
+      <c r="E23" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>169</v>
+      </c>
+      <c r="C24" t="s">
+        <v>170</v>
+      </c>
+      <c r="D24" t="s">
+        <v>171</v>
+      </c>
+      <c r="E24" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" t="s">
+        <v>173</v>
+      </c>
+      <c r="D25" t="s">
+        <v>174</v>
+      </c>
+      <c r="E25" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" t="s">
+        <v>177</v>
+      </c>
+      <c r="E26" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" t="s">
+        <v>180</v>
+      </c>
+      <c r="D27" t="s">
+        <v>181</v>
+      </c>
+      <c r="E27" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>183</v>
+      </c>
+      <c r="C28" t="s">
+        <v>184</v>
+      </c>
+      <c r="D28" t="s">
+        <v>185</v>
+      </c>
+      <c r="E28" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>187</v>
+      </c>
+      <c r="C29" t="s">
+        <v>188</v>
+      </c>
+      <c r="D29" t="s">
+        <v>189</v>
+      </c>
+      <c r="E29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" t="s">
+        <v>192</v>
+      </c>
+      <c r="D30" t="s">
+        <v>193</v>
+      </c>
+      <c r="E30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>194</v>
+      </c>
+      <c r="C31" t="s">
+        <v>195</v>
+      </c>
+      <c r="D31" t="s">
+        <v>196</v>
+      </c>
+      <c r="E31" t="s">
+        <v>197</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC2FCC6C-2415-4358-BDD7-E21BEB1CA86A}">
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.109375" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="19.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" customWidth="1"/>
+    <col min="6" max="6" width="37" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" t="s">
+        <v>229</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" t="s">
+        <v>213</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" t="s">
+        <v>214</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>203</v>
+      </c>
+      <c r="B12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>203</v>
+      </c>
+      <c r="B13" t="s">
+        <v>231</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" t="s">
+        <v>232</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B15" t="s">
+        <v>342</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" t="s">
+        <v>216</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>203</v>
+      </c>
+      <c r="B17" t="s">
+        <v>217</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>203</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>203</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>203</v>
+      </c>
+      <c r="B20" t="s">
+        <v>218</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" t="s">
+        <v>219</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>203</v>
+      </c>
+      <c r="B22" t="s">
+        <v>215</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B23" t="s">
+        <v>220</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>203</v>
+      </c>
+      <c r="B24" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>203</v>
+      </c>
+      <c r="B25" t="s">
+        <v>222</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>203</v>
+      </c>
+      <c r="B26" t="s">
+        <v>223</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>203</v>
+      </c>
+      <c r="B27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>203</v>
+      </c>
+      <c r="B28" t="s">
+        <v>225</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>203</v>
+      </c>
+      <c r="B29" t="s">
+        <v>226</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>203</v>
+      </c>
+      <c r="B30" t="s">
+        <v>227</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>203</v>
+      </c>
+      <c r="B31" t="s">
+        <v>228</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>203</v>
+      </c>
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>203</v>
+      </c>
+      <c r="B33" t="s">
+        <v>337</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>204</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>204</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>204</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>204</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>204</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>204</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>204</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>204</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>204</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>204</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>204</v>
+      </c>
+      <c r="B45" t="s">
+        <v>30</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>204</v>
+      </c>
+      <c r="B46" t="s">
+        <v>337</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>205</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>205</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>205</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D49" s="6"/>
+      <c r="E49" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="G50" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="C51" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="G51" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>205</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>205</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>205</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>205</v>
+      </c>
+      <c r="B55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>205</v>
+      </c>
+      <c r="B56" t="s">
+        <v>337</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>206</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>206</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>206</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>206</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B62" t="s">
+        <v>30</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D62" s="6"/>
+      <c r="E62" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B63" t="s">
+        <v>337</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B71" t="s">
+        <v>30</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B72" t="s">
+        <v>337</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BCA21BD-59C0-4361-BACF-2FAAB2258582}">
   <dimension ref="A1:AD6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="2"/>
-    <col min="4" max="5" width="11.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.88671875" style="2"/>
-    <col min="9" max="9" width="4.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="3.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="8.88671875" style="2"/>
-    <col min="21" max="21" width="4.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="4.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.88671875" style="2"/>
-    <col min="26" max="26" width="8.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.88671875" style="2"/>
-    <col min="28" max="28" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1">
         <v>5.0999999999999996</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" s="1">
         <v>1783354551905</v>
@@ -786,10 +3591,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I2" s="1">
         <v>38</v>
@@ -800,7 +3605,7 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N2" s="1">
         <v>0</v>
@@ -809,19 +3614,19 @@
         <v>415</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="U2" s="1">
         <v>63</v>
@@ -836,13 +3641,13 @@
         <v>68</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AB2" s="1">
         <v>-71.825199999999995</v>
@@ -856,13 +3661,13 @@
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" s="1">
         <v>5.0999999999999996</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D3" s="1">
         <v>1783349018525</v>
@@ -872,17 +3677,17 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N3" s="1">
         <v>0</v>
@@ -891,19 +3696,19 @@
         <v>400</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="U3" s="1">
         <v>29</v>
@@ -918,13 +3723,13 @@
         <v>68</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AB3" s="1">
         <v>-172.07</v>
@@ -938,13 +3743,13 @@
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B4" s="1">
         <v>5.4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" s="1">
         <v>1783327298715</v>
@@ -954,10 +3759,10 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I4" s="1">
         <v>2</v>
@@ -969,10 +3774,10 @@
         <v>3.9489999999999998</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N4" s="1">
         <v>0</v>
@@ -981,19 +3786,19 @@
         <v>449</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U4" s="1">
         <v>66</v>
@@ -1008,13 +3813,13 @@
         <v>41</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AB4" s="1">
         <v>125.14239999999999</v>
@@ -1028,13 +3833,13 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1">
         <v>5.8</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" s="1">
         <v>1783325471032</v>
@@ -1044,10 +3849,10 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I5" s="1">
         <v>7</v>
@@ -1059,10 +3864,10 @@
         <v>4.3289999999999997</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N5" s="1">
         <v>0</v>
@@ -1071,19 +3876,19 @@
         <v>521</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="U5" s="1">
         <v>78</v>
@@ -1098,13 +3903,13 @@
         <v>37</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AB5" s="1">
         <v>125.32599999999999</v>
@@ -1118,13 +3923,13 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B6" s="1">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D6" s="1">
         <v>1783266813718</v>
@@ -1134,17 +3939,17 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N6" s="1">
         <v>0</v>
@@ -1153,19 +3958,19 @@
         <v>385</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="U6" s="1">
         <v>59</v>
@@ -1180,13 +3985,13 @@
         <v>106</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AB6" s="1">
         <v>-72.011300000000006</v>

</xml_diff>

<commit_message>
Model finished and tests added
</commit_message>
<xml_diff>
--- a/model_analysis.xlsx
+++ b/model_analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EdwardCoates\Dev\snowflake_sandbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C97D4CDE-1D4E-4354-ADEC-41BCD49F6EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EC3027-EFCE-47F2-BCE0-FC78A1A9A0B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{0818FD26-D4B8-4367-BAC1-03867A914A11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{0818FD26-D4B8-4367-BAC1-03867A914A11}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Data Dictionary" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="349">
   <si>
     <t>ID</t>
   </si>
@@ -897,18 +897,9 @@
     <t>PAGER_ALERT_RANK</t>
   </si>
   <si>
-    <t>REVIEW_STATUS</t>
-  </si>
-  <si>
-    <t>IS_REVIEWED</t>
-  </si>
-  <si>
     <t>TSUNAMI_FLAG</t>
   </si>
   <si>
-    <t>HAS_FELT_REPORTS</t>
-  </si>
-  <si>
     <t>INTEGER</t>
   </si>
   <si>
@@ -918,18 +909,6 @@
     <t>Ordinal 0–4 for sorting/severity.</t>
   </si>
   <si>
-    <t>automatic / reviewed (STATUS).</t>
-  </si>
-  <si>
-    <t>True when reviewed by a human.</t>
-  </si>
-  <si>
-    <t>True when TSUNAMI = 1.</t>
-  </si>
-  <si>
-    <t>True when FELT is present and &gt; 0.</t>
-  </si>
-  <si>
     <t>Surrogate key for each flag combination.</t>
   </si>
   <si>
@@ -1096,6 +1075,24 @@
   </si>
   <si>
     <t>Column1</t>
+  </si>
+  <si>
+    <t>REVIEWED_BY_HUMAN_FLAG</t>
+  </si>
+  <si>
+    <t>Y when reviewed by a human.</t>
+  </si>
+  <si>
+    <t>Y when TSUNAMI = 1.</t>
+  </si>
+  <si>
+    <t>Y when FELT is present and &gt; 0.</t>
+  </si>
+  <si>
+    <t>FELT_BY_HUMAN_FLAG</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
 </sst>
 </file>
@@ -1184,7 +1181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1213,7 +1210,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1299,8 +1295,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}" name="Table3" displayName="Table3" ref="A8:G72" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A8:G72" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}" name="Table3" displayName="Table3" ref="A8:G71" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A8:G71" xr:uid="{11930668-30EA-4F9B-8CC8-ECD9874A4EDC}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{5D127818-973C-4145-B700-33EA8DCCBA9C}" name="Table"/>
     <tableColumn id="2" xr3:uid="{64F6B203-BA28-42A1-8A8E-83B001CBB1A7}" name="Column"/>
@@ -1632,16 +1628,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1A630FB-A618-42DB-96FD-BC7A66867678}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="93.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="89.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="93.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="89.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>198</v>
       </c>
@@ -1658,7 +1654,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1675,7 +1671,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1692,7 +1688,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1709,7 +1705,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1726,7 +1722,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1743,7 +1739,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1760,7 +1756,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1777,7 +1773,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1794,7 +1790,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1811,7 +1807,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1828,7 +1824,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1845,7 +1841,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1862,7 +1858,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1879,7 +1875,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1896,7 +1892,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1913,7 +1909,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1930,7 +1926,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1947,7 +1943,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1964,7 +1960,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1981,7 +1977,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1998,7 +1994,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -2015,7 +2011,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2032,7 +2028,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -2049,7 +2045,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -2066,7 +2062,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -2083,7 +2079,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -2100,7 +2096,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -2117,7 +2113,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -2134,7 +2130,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -2151,7 +2147,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -2178,17 +2174,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC2FCC6C-2415-4358-BDD7-E21BEB1CA86A}">
-  <dimension ref="A1:G72"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.109375" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.88671875" customWidth="1"/>
+    <col min="1" max="1" width="27.08984375" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="19.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>201</v>
       </c>
@@ -2196,7 +2192,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>203</v>
       </c>
@@ -2204,7 +2200,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>204</v>
       </c>
@@ -2212,7 +2208,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>205</v>
       </c>
@@ -2220,7 +2216,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>206</v>
       </c>
@@ -2228,7 +2224,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>207</v>
       </c>
@@ -2236,7 +2232,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>201</v>
       </c>
@@ -2247,7 +2243,7 @@
         <v>79</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>80</v>
@@ -2255,11 +2251,11 @@
       <c r="F8" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="G8" s="12" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G8" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>203</v>
       </c>
@@ -2273,13 +2269,13 @@
         <v>234</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>203</v>
       </c>
@@ -2290,16 +2286,16 @@
         <v>239</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>203</v>
       </c>
@@ -2311,13 +2307,13 @@
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>203</v>
       </c>
@@ -2327,15 +2323,17 @@
       <c r="C12" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="E12" s="6" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>203</v>
       </c>
@@ -2345,15 +2343,17 @@
       <c r="C13" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="E13" s="6" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>203</v>
       </c>
@@ -2363,33 +2363,35 @@
       <c r="C14" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D14" s="6"/>
+      <c r="D14" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="E14" s="6" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>203</v>
       </c>
       <c r="B15" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>203</v>
       </c>
@@ -2401,13 +2403,13 @@
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>203</v>
       </c>
@@ -2419,13 +2421,13 @@
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>203</v>
       </c>
@@ -2433,17 +2435,17 @@
         <v>28</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>203</v>
       </c>
@@ -2451,17 +2453,17 @@
         <v>27</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>203</v>
       </c>
@@ -2469,17 +2471,17 @@
         <v>218</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>203</v>
       </c>
@@ -2487,17 +2489,17 @@
         <v>219</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>203</v>
       </c>
@@ -2509,13 +2511,13 @@
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>203</v>
       </c>
@@ -2523,17 +2525,17 @@
         <v>220</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>203</v>
       </c>
@@ -2545,13 +2547,13 @@
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>203</v>
       </c>
@@ -2559,17 +2561,17 @@
         <v>222</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>203</v>
       </c>
@@ -2577,17 +2579,17 @@
         <v>223</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>203</v>
       </c>
@@ -2599,13 +2601,13 @@
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>203</v>
       </c>
@@ -2617,13 +2619,13 @@
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>203</v>
       </c>
@@ -2631,17 +2633,17 @@
         <v>226</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>203</v>
       </c>
@@ -2649,17 +2651,17 @@
         <v>227</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>203</v>
       </c>
@@ -2667,17 +2669,17 @@
         <v>228</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>203</v>
       </c>
@@ -2685,35 +2687,35 @@
         <v>30</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>203</v>
       </c>
       <c r="B33" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>204</v>
       </c>
@@ -2733,7 +2735,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>204</v>
       </c>
@@ -2751,7 +2753,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>204</v>
       </c>
@@ -2769,7 +2771,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>204</v>
       </c>
@@ -2787,7 +2789,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>204</v>
       </c>
@@ -2805,7 +2807,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>204</v>
       </c>
@@ -2823,7 +2825,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>204</v>
       </c>
@@ -2841,7 +2843,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>204</v>
       </c>
@@ -2859,7 +2861,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>204</v>
       </c>
@@ -2877,7 +2879,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>204</v>
       </c>
@@ -2895,7 +2897,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>204</v>
       </c>
@@ -2913,7 +2915,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>204</v>
       </c>
@@ -2921,35 +2923,35 @@
         <v>30</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>204</v>
       </c>
       <c r="B46" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>205</v>
       </c>
@@ -2969,12 +2971,12 @@
         <v>261</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>205</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>239</v>
@@ -2987,12 +2989,12 @@
         <v>262</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>205</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>239</v>
@@ -3005,7 +3007,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>205</v>
       </c>
@@ -3023,15 +3025,15 @@
         <v>264</v>
       </c>
       <c r="G50" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>205</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>239</v>
@@ -3044,10 +3046,10 @@
         <v>264</v>
       </c>
       <c r="G51" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>205</v>
       </c>
@@ -3065,7 +3067,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>205</v>
       </c>
@@ -3083,7 +3085,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>205</v>
       </c>
@@ -3094,7 +3096,7 @@
         <v>239</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>236</v>
@@ -3103,7 +3105,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>205</v>
       </c>
@@ -3111,35 +3113,35 @@
         <v>30</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>205</v>
       </c>
       <c r="B56" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>206</v>
       </c>
@@ -3147,7 +3149,7 @@
         <v>231</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>234</v>
@@ -3159,7 +3161,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>206</v>
       </c>
@@ -3170,7 +3172,7 @@
         <v>239</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>236</v>
@@ -3179,7 +3181,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>206</v>
       </c>
@@ -3190,7 +3192,7 @@
         <v>239</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>236</v>
@@ -3199,7 +3201,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>206</v>
       </c>
@@ -3217,7 +3219,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
         <v>206</v>
       </c>
@@ -3228,7 +3230,7 @@
         <v>239</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>236</v>
@@ -3237,7 +3239,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
         <v>206</v>
       </c>
@@ -3245,35 +3247,35 @@
         <v>30</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
         <v>206</v>
       </c>
       <c r="B63" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
         <v>207</v>
       </c>
@@ -3290,10 +3292,10 @@
         <v>234</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
         <v>207</v>
       </c>
@@ -3304,16 +3306,16 @@
         <v>239</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>236</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>207</v>
       </c>
@@ -3328,121 +3330,101 @@
         <v>236</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>283</v>
+        <v>343</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>346</v>
-      </c>
+        <v>265</v>
+      </c>
+      <c r="D67" s="6"/>
       <c r="E67" s="6" t="s">
         <v>236</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="D68" s="6"/>
+        <v>265</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="E68" s="6" t="s">
         <v>236</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>285</v>
+        <v>347</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>242</v>
+        <v>265</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>236</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>286</v>
+      <c r="B70" t="s">
+        <v>30</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="D70" s="6" t="s">
-        <v>346</v>
-      </c>
+        <v>331</v>
+      </c>
+      <c r="D70" s="6"/>
       <c r="E70" s="6" t="s">
-        <v>236</v>
+        <v>334</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B71" t="s">
-        <v>30</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="D71" s="6"/>
-      <c r="E71" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="F71" s="6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B72" t="s">
-        <v>337</v>
-      </c>
-      <c r="C72" s="8" t="s">
-        <v>338</v>
-      </c>
-      <c r="D72" s="8"/>
-      <c r="E72" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="F72" s="8" t="s">
-        <v>340</v>
+        <v>330</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="D71" s="8"/>
+      <c r="E71" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="F71" s="8" t="s">
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -3456,32 +3438,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BCA21BD-59C0-4361-BACF-2FAAB2258582}">
   <dimension ref="A1:AD6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="3.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.54296875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="4.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3573,7 +3555,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -3659,7 +3641,7 @@
         <v>20.998000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -3741,7 +3723,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>53</v>
       </c>
@@ -3831,7 +3813,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>62</v>
       </c>
@@ -3921,7 +3903,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>71</v>
       </c>

</xml_diff>